<commit_message>
upload excel data indikator & sasaran awal di pegawai
</commit_message>
<xml_diff>
--- a/uploads/Template_UploadDataIndikator_Perunit_jabatan.xlsx
+++ b/uploads/Template_UploadDataIndikator_Perunit_jabatan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Laragon\laragon\www\SKI-BRK\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E803B1-BE4E-40E3-9191-50A09CBBC038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFBE054-88F7-474F-9242-1A4DBCAB5BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{AFB8C1B9-0976-4362-9026-160F0EE58800}"/>
+    <workbookView xWindow="3480" yWindow="3830" windowWidth="14400" windowHeight="8170" xr2:uid="{AFB8C1B9-0976-4362-9026-160F0EE58800}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -170,7 +170,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -641,7 +641,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -711,7 +711,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -735,31 +735,139 @@
       <alignment wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="33" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="33" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="38" fontId="1" fillId="0" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="2" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -783,6 +891,34 @@
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -790,31 +926,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -822,23 +934,11 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -858,133 +958,32 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="38" fontId="1" fillId="0" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -1305,56 +1304,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045A5E13-C48B-45B7-B96B-940681A75227}">
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:14" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="57" t="s">
+      <c r="B1" s="45"/>
+      <c r="C1" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="59"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="48"/>
       <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="60" t="s">
+      <c r="H1" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="56"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="45"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="63" t="s">
+      <c r="B2" s="51"/>
+      <c r="C2" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="62"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="51"/>
       <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="H2" s="3"/>
-      <c r="I2" s="65" t="s">
+      <c r="I2" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="65"/>
-      <c r="M2" s="65"/>
-      <c r="N2" s="66"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
+      <c r="N2" s="55"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
@@ -1370,486 +1369,483 @@
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
-      <c r="N3" s="67"/>
+      <c r="N3" s="25"/>
     </row>
     <row r="4" spans="1:14" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="38"/>
+      <c r="B4" s="65"/>
       <c r="C4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="74" t="s">
+      <c r="D4" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="74"/>
-      <c r="F4" s="75"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="29"/>
       <c r="G4" s="7"/>
       <c r="H4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-      <c r="M4" s="39"/>
-      <c r="N4" s="40"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="56"/>
+      <c r="M4" s="56"/>
+      <c r="N4" s="57"/>
     </row>
     <row r="5" spans="1:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="86"/>
-      <c r="B5" s="47"/>
+      <c r="A5" s="66"/>
+      <c r="B5" s="67"/>
       <c r="C5" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
-      <c r="F5" s="75"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="29"/>
       <c r="G5" s="7"/>
       <c r="H5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="72"/>
-      <c r="J5" s="72"/>
-      <c r="K5" s="72"/>
-      <c r="L5" s="72"/>
-      <c r="M5" s="72"/>
-      <c r="N5" s="73"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="33"/>
+      <c r="N5" s="34"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="33"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="60"/>
       <c r="G6" s="9">
         <f>SUM(G4:G4)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="34" t="s">
+      <c r="H6" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="35"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="35"/>
-      <c r="L6" s="35"/>
-      <c r="M6" s="35"/>
-      <c r="N6" s="36"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
+      <c r="K6" s="62"/>
+      <c r="L6" s="62"/>
+      <c r="M6" s="62"/>
+      <c r="N6" s="63"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="71" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="38"/>
-      <c r="C7" s="41" t="s">
+      <c r="B7" s="65"/>
+      <c r="C7" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="44" t="s">
+      <c r="D7" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="44"/>
-      <c r="F7" s="38"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="65"/>
       <c r="G7" s="7">
         <v>5</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="51" t="s">
+      <c r="I7" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="51"/>
-      <c r="K7" s="51"/>
-      <c r="L7" s="51"/>
-      <c r="M7" s="51"/>
-      <c r="N7" s="52"/>
+      <c r="J7" s="76"/>
+      <c r="K7" s="76"/>
+      <c r="L7" s="76"/>
+      <c r="M7" s="76"/>
+      <c r="N7" s="77"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A8" s="48"/>
-      <c r="B8" s="45"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="45"/>
+      <c r="A8" s="72"/>
+      <c r="B8" s="73"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="75"/>
+      <c r="E8" s="75"/>
+      <c r="F8" s="73"/>
       <c r="G8" s="7">
         <v>5</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="53" t="s">
+      <c r="I8" s="78" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="53"/>
-      <c r="K8" s="53"/>
-      <c r="L8" s="53"/>
-      <c r="M8" s="53"/>
-      <c r="N8" s="54"/>
+      <c r="J8" s="78"/>
+      <c r="K8" s="78"/>
+      <c r="L8" s="78"/>
+      <c r="M8" s="78"/>
+      <c r="N8" s="79"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A9" s="48"/>
-      <c r="B9" s="45"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="47"/>
-      <c r="G9" s="7">
-        <v>10</v>
-      </c>
+      <c r="A9" s="72"/>
+      <c r="B9" s="73"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="67"/>
+      <c r="G9" s="7"/>
       <c r="H9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="53"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
-      <c r="M9" s="53"/>
-      <c r="N9" s="54"/>
+      <c r="I9" s="78"/>
+      <c r="J9" s="78"/>
+      <c r="K9" s="78"/>
+      <c r="L9" s="78"/>
+      <c r="M9" s="78"/>
+      <c r="N9" s="79"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A10" s="48"/>
-      <c r="B10" s="45"/>
-      <c r="C10" s="41" t="s">
+      <c r="A10" s="72"/>
+      <c r="B10" s="73"/>
+      <c r="C10" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="44" t="s">
+      <c r="D10" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="44"/>
-      <c r="F10" s="38"/>
+      <c r="E10" s="68"/>
+      <c r="F10" s="65"/>
       <c r="G10" s="7">
         <v>10</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="39" t="s">
+      <c r="I10" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="39"/>
-      <c r="K10" s="39"/>
-      <c r="L10" s="39"/>
-      <c r="M10" s="39"/>
-      <c r="N10" s="40"/>
+      <c r="J10" s="56"/>
+      <c r="K10" s="56"/>
+      <c r="L10" s="56"/>
+      <c r="M10" s="56"/>
+      <c r="N10" s="57"/>
     </row>
     <row r="11" spans="1:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="49"/>
-      <c r="B11" s="47"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="47"/>
+      <c r="A11" s="74"/>
+      <c r="B11" s="67"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="67"/>
       <c r="G11" s="7">
         <v>10</v>
       </c>
-      <c r="H11" s="83" t="s">
+      <c r="H11" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="39" t="s">
+      <c r="I11" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="J11" s="39"/>
-      <c r="K11" s="39"/>
-      <c r="L11" s="39"/>
-      <c r="M11" s="39"/>
-      <c r="N11" s="40"/>
+      <c r="J11" s="56"/>
+      <c r="K11" s="56"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="56"/>
+      <c r="N11" s="57"/>
     </row>
     <row r="12" spans="1:14" ht="31" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="70"/>
-      <c r="B12" s="71"/>
+      <c r="A12" s="42"/>
+      <c r="B12" s="43"/>
       <c r="C12" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
-      <c r="F12" s="75"/>
-      <c r="G12" s="82"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="26"/>
       <c r="H12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I12" s="72"/>
-      <c r="J12" s="72"/>
-      <c r="K12" s="72"/>
-      <c r="L12" s="72"/>
-      <c r="M12" s="72"/>
-      <c r="N12" s="73"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="33"/>
+      <c r="M12" s="33"/>
+      <c r="N12" s="34"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="33"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="59"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="60"/>
       <c r="G13" s="9">
         <f>SUM(G7:G11)</f>
-        <v>40</v>
-      </c>
-      <c r="H13" s="84" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="70" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="35"/>
-      <c r="L13" s="35"/>
-      <c r="M13" s="35"/>
-      <c r="N13" s="36"/>
+      <c r="I13" s="62"/>
+      <c r="J13" s="62"/>
+      <c r="K13" s="62"/>
+      <c r="L13" s="62"/>
+      <c r="M13" s="62"/>
+      <c r="N13" s="63"/>
     </row>
     <row r="14" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="79" t="s">
+      <c r="A14" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="75"/>
-      <c r="C14" s="41" t="s">
+      <c r="B14" s="29"/>
+      <c r="C14" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="74" t="s">
+      <c r="D14" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="74"/>
-      <c r="F14" s="75"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="29"/>
       <c r="G14" s="7">
         <v>10</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I14" s="39" t="s">
+      <c r="I14" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="J14" s="39"/>
-      <c r="K14" s="39"/>
-      <c r="L14" s="39"/>
-      <c r="M14" s="39"/>
-      <c r="N14" s="40"/>
+      <c r="J14" s="56"/>
+      <c r="K14" s="56"/>
+      <c r="L14" s="56"/>
+      <c r="M14" s="56"/>
+      <c r="N14" s="57"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A15" s="80"/>
-      <c r="B15" s="81"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="87"/>
-      <c r="E15" s="87"/>
-      <c r="F15" s="81"/>
+      <c r="A15" s="40"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="36"/>
       <c r="G15" s="7">
         <v>5</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="39" t="s">
+      <c r="I15" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="J15" s="39"/>
-      <c r="K15" s="39"/>
-      <c r="L15" s="39"/>
-      <c r="M15" s="39"/>
-      <c r="N15" s="40"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="56"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="56"/>
+      <c r="N15" s="57"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A16" s="80"/>
-      <c r="B16" s="81"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="76"/>
-      <c r="E16" s="76"/>
-      <c r="F16" s="77"/>
+      <c r="A16" s="40"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="38"/>
       <c r="G16" s="7"/>
       <c r="H16" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I16" s="39"/>
-      <c r="J16" s="39"/>
-      <c r="K16" s="39"/>
-      <c r="L16" s="39"/>
-      <c r="M16" s="39"/>
-      <c r="N16" s="40"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A17" s="80"/>
-      <c r="B17" s="81"/>
-      <c r="C17" s="41" t="s">
+      <c r="I16" s="56"/>
+      <c r="J16" s="56"/>
+      <c r="K16" s="56"/>
+      <c r="L16" s="56"/>
+      <c r="M16" s="56"/>
+      <c r="N16" s="57"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A17" s="40"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="44" t="s">
+      <c r="D17" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="44"/>
-      <c r="F17" s="38"/>
+      <c r="E17" s="68"/>
+      <c r="F17" s="65"/>
       <c r="G17" s="11">
         <v>15</v>
       </c>
       <c r="H17" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I17" s="39" t="s">
+      <c r="I17" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="J17" s="39"/>
-      <c r="K17" s="39"/>
-      <c r="L17" s="39"/>
-      <c r="M17" s="39"/>
-      <c r="N17" s="40"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A18" s="80"/>
-      <c r="B18" s="81"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="68"/>
-      <c r="E18" s="68"/>
-      <c r="F18" s="45"/>
+      <c r="J17" s="56"/>
+      <c r="K17" s="56"/>
+      <c r="L17" s="56"/>
+      <c r="M17" s="56"/>
+      <c r="N17" s="57"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A18" s="40"/>
+      <c r="B18" s="36"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="75"/>
+      <c r="E18" s="75"/>
+      <c r="F18" s="73"/>
       <c r="G18" s="11">
         <v>5</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="39" t="s">
+      <c r="I18" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="J18" s="39"/>
-      <c r="K18" s="39"/>
-      <c r="L18" s="39"/>
-      <c r="M18" s="39"/>
-      <c r="N18" s="40"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A19" s="80"/>
-      <c r="B19" s="81"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="46"/>
-      <c r="E19" s="46"/>
-      <c r="F19" s="47"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="56"/>
+      <c r="M18" s="56"/>
+      <c r="N18" s="57"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A19" s="40"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="69"/>
+      <c r="F19" s="67"/>
       <c r="G19" s="7"/>
       <c r="H19" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I19" s="39"/>
-      <c r="J19" s="39"/>
-      <c r="K19" s="39"/>
-      <c r="L19" s="39"/>
-      <c r="M19" s="39"/>
-      <c r="N19" s="40"/>
-      <c r="P19" s="85"/>
-    </row>
-    <row r="20" spans="1:16" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="78"/>
-      <c r="B20" s="77"/>
+      <c r="I19" s="56"/>
+      <c r="J19" s="56"/>
+      <c r="K19" s="56"/>
+      <c r="L19" s="56"/>
+      <c r="M19" s="56"/>
+      <c r="N19" s="57"/>
+    </row>
+    <row r="20" spans="1:14" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="41"/>
+      <c r="B20" s="38"/>
       <c r="C20" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="74"/>
-      <c r="E20" s="74"/>
-      <c r="F20" s="75"/>
-      <c r="G20" s="82"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="26"/>
       <c r="H20" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="I20" s="72"/>
-      <c r="J20" s="72"/>
-      <c r="K20" s="72"/>
-      <c r="L20" s="72"/>
-      <c r="M20" s="72"/>
-      <c r="N20" s="73"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A21" s="31" t="s">
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="33"/>
+      <c r="N20" s="34"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A21" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="33"/>
+      <c r="B21" s="59"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="60"/>
       <c r="G21" s="9">
         <f>SUM(G14:G19)</f>
         <v>35</v>
       </c>
-      <c r="H21" s="34" t="s">
+      <c r="H21" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="35"/>
-      <c r="M21" s="35"/>
-      <c r="N21" s="36"/>
-    </row>
-    <row r="22" spans="1:16" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="44" t="s">
+      <c r="I21" s="62"/>
+      <c r="J21" s="62"/>
+      <c r="K21" s="62"/>
+      <c r="L21" s="62"/>
+      <c r="M21" s="62"/>
+      <c r="N21" s="63"/>
+    </row>
+    <row r="22" spans="1:14" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="38"/>
+      <c r="B22" s="65"/>
       <c r="C22" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="74" t="s">
+      <c r="D22" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="74"/>
-      <c r="F22" s="75"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="29"/>
       <c r="G22" s="12">
         <v>5</v>
       </c>
       <c r="H22" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I22" s="72" t="s">
+      <c r="I22" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="J22" s="72"/>
-      <c r="K22" s="72"/>
-      <c r="L22" s="72"/>
-      <c r="M22" s="72"/>
-      <c r="N22" s="73"/>
-    </row>
-    <row r="23" spans="1:16" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="46"/>
-      <c r="B23" s="47"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+      <c r="N22" s="34"/>
+    </row>
+    <row r="23" spans="1:14" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="69"/>
+      <c r="B23" s="67"/>
       <c r="C23" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="74"/>
-      <c r="E23" s="74"/>
-      <c r="F23" s="75"/>
-      <c r="G23" s="82"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="26"/>
       <c r="H23" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I23" s="72"/>
-      <c r="J23" s="72"/>
-      <c r="K23" s="72"/>
-      <c r="L23" s="72"/>
-      <c r="M23" s="72"/>
-      <c r="N23" s="73"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A24" s="31" t="s">
+      <c r="I23" s="33"/>
+      <c r="J23" s="33"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="33"/>
+      <c r="N23" s="34"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A24" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="32"/>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="33"/>
+      <c r="B24" s="59"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="60"/>
       <c r="G24" s="9">
         <f>SUM(G22:G22)</f>
         <v>5</v>
       </c>
-      <c r="H24" s="34" t="s">
+      <c r="H24" s="61" t="s">
         <v>38</v>
       </c>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35"/>
-      <c r="K24" s="35"/>
-      <c r="L24" s="35"/>
-      <c r="M24" s="35"/>
-      <c r="N24" s="36"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I24" s="62"/>
+      <c r="J24" s="62"/>
+      <c r="K24" s="62"/>
+      <c r="L24" s="62"/>
+      <c r="M24" s="62"/>
+      <c r="N24" s="63"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" s="4"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1863,9 +1859,9 @@
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
-      <c r="N25" s="67"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="N25" s="25"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" s="14"/>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -1874,37 +1870,37 @@
       <c r="F26" s="16"/>
       <c r="G26" s="17"/>
       <c r="H26" s="18"/>
-      <c r="I26" s="25"/>
-      <c r="J26" s="25"/>
-      <c r="K26" s="25"/>
-      <c r="L26" s="25"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="26"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A27" s="27" t="s">
+      <c r="I26" s="80"/>
+      <c r="J26" s="80"/>
+      <c r="K26" s="80"/>
+      <c r="L26" s="80"/>
+      <c r="M26" s="80"/>
+      <c r="N26" s="81"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A27" s="82" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="69"/>
-      <c r="C27" s="69"/>
-      <c r="D27" s="69"/>
-      <c r="E27" s="69"/>
-      <c r="F27" s="28"/>
+      <c r="B27" s="83"/>
+      <c r="C27" s="83"/>
+      <c r="D27" s="83"/>
+      <c r="E27" s="83"/>
+      <c r="F27" s="84"/>
       <c r="G27" s="19">
         <f>G6+G13+G21+G24</f>
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H27" s="20"/>
-      <c r="I27" s="69" t="s">
+      <c r="I27" s="83" t="s">
         <v>40</v>
       </c>
-      <c r="J27" s="69"/>
-      <c r="K27" s="69"/>
-      <c r="L27" s="69"/>
-      <c r="M27" s="69"/>
-      <c r="N27" s="28"/>
-    </row>
-    <row r="28" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="J27" s="83"/>
+      <c r="K27" s="83"/>
+      <c r="L27" s="83"/>
+      <c r="M27" s="83"/>
+      <c r="N27" s="84"/>
+    </row>
+    <row r="28" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="21"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -1913,59 +1909,15 @@
       <c r="F28" s="23"/>
       <c r="G28" s="24"/>
       <c r="H28" s="24"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="29"/>
-      <c r="L28" s="29"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="30"/>
+      <c r="I28" s="85"/>
+      <c r="J28" s="85"/>
+      <c r="K28" s="85"/>
+      <c r="L28" s="85"/>
+      <c r="M28" s="85"/>
+      <c r="N28" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="I22:N22"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="D14:F16"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A14:B20"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="I12:N12"/>
-    <mergeCell ref="I20:N20"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="H1:N1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="I2:N2"/>
-    <mergeCell ref="I4:N4"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:N6"/>
-    <mergeCell ref="A4:B5"/>
-    <mergeCell ref="I5:N5"/>
-    <mergeCell ref="I14:N14"/>
-    <mergeCell ref="I15:N15"/>
-    <mergeCell ref="D10:F11"/>
-    <mergeCell ref="I10:N10"/>
-    <mergeCell ref="I11:N11"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="H13:N13"/>
-    <mergeCell ref="A7:B11"/>
-    <mergeCell ref="D7:F9"/>
-    <mergeCell ref="I7:N7"/>
-    <mergeCell ref="I8:N8"/>
-    <mergeCell ref="I9:N9"/>
-    <mergeCell ref="I16:N16"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="D17:F19"/>
-    <mergeCell ref="I17:N17"/>
-    <mergeCell ref="I18:N18"/>
-    <mergeCell ref="I19:N19"/>
     <mergeCell ref="I26:N26"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="I27:N27"/>
@@ -1976,6 +1928,50 @@
     <mergeCell ref="H24:N24"/>
     <mergeCell ref="A22:B23"/>
     <mergeCell ref="I23:N23"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="I16:N16"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="D17:F19"/>
+    <mergeCell ref="I17:N17"/>
+    <mergeCell ref="I18:N18"/>
+    <mergeCell ref="I19:N19"/>
+    <mergeCell ref="I4:N4"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:N6"/>
+    <mergeCell ref="A4:B5"/>
+    <mergeCell ref="I5:N5"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:F1"/>
+    <mergeCell ref="H1:N1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="I2:N2"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A14:B20"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D10:F11"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A7:B11"/>
+    <mergeCell ref="D7:F9"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="I22:N22"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="D14:F16"/>
+    <mergeCell ref="I12:N12"/>
+    <mergeCell ref="I20:N20"/>
+    <mergeCell ref="I14:N14"/>
+    <mergeCell ref="I15:N15"/>
+    <mergeCell ref="I10:N10"/>
+    <mergeCell ref="I11:N11"/>
+    <mergeCell ref="H13:N13"/>
+    <mergeCell ref="I7:N7"/>
+    <mergeCell ref="I8:N8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>